<commit_message>
feat: scaffold full-stack wishes application with wizard, dashboard, and automation services
</commit_message>
<xml_diff>
--- a/public/demo.xlsx
+++ b/public/demo.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Events" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E51"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,70 +414,868 @@
         <v>Email</v>
       </c>
       <c r="C1" t="str">
-        <v>PhotoURL</v>
+        <v>Department</v>
       </c>
       <c r="D1" t="str">
-        <v>EventType</v>
+        <v>Occasion</v>
       </c>
       <c r="E1" t="str">
         <v>EventDate</v>
       </c>
-      <c r="F1" t="str">
-        <v>Department</v>
-      </c>
-      <c r="G1" t="str">
-        <v>CustomMessage</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Kamalesh</v>
+        <v>Sarah Johnson</v>
       </c>
       <c r="B2" t="str">
-        <v>kamalesh@example.com</v>
+        <v>sarah.johnson@company.com</v>
       </c>
       <c r="C2" t="str">
-        <v>https://images.unsplash.com/photo-1535713875002-d1d0cf377fde</v>
+        <v>Sales</v>
       </c>
       <c r="D2" t="str">
-        <v>Birthday</v>
+        <v>Work Anniversary</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-07-20</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Engineering</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Happy Birthday Kamalesh! Have a fantastic day ahead!</v>
+        <v>2026-09-11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sang</v>
+        <v>Charles Smith</v>
       </c>
       <c r="B3" t="str">
-        <v>sang@example.com</v>
+        <v>charles.smith@company.com</v>
       </c>
       <c r="C3" t="str">
-        <v>https://images.unsplash.com/photo-1494790108377-be9c29b29330</v>
+        <v>Design</v>
       </c>
       <c r="D3" t="str">
-        <v>Anniversary</v>
+        <v>Work Anniversary</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-10-15</v>
-      </c>
-      <c r="F3" t="str">
+        <v>2026-08-26</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Sarah Anderson</v>
+      </c>
+      <c r="B4" t="str">
+        <v>sarah.anderson@company.com</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-06-20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Susan Hernandez</v>
+      </c>
+      <c r="B5" t="str">
+        <v>susan.hernandez@company.com</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-02-08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>William Williams</v>
+      </c>
+      <c r="B6" t="str">
+        <v>william.williams@company.com</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-11-13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Robert Johnson</v>
+      </c>
+      <c r="B7" t="str">
+        <v>robert.johnson@company.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-10-13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Karen Jones</v>
+      </c>
+      <c r="B8" t="str">
+        <v>karen.jones@company.com</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-11-22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>John Lopez</v>
+      </c>
+      <c r="B9" t="str">
+        <v>john.lopez@company.com</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-04-04</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Thomas Moore</v>
+      </c>
+      <c r="B10" t="str">
+        <v>thomas.moore@company.com</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-01-23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Linda Smith</v>
+      </c>
+      <c r="B11" t="str">
+        <v>linda.smith@company.com</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-09-02</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Linda Johnson</v>
+      </c>
+      <c r="B12" t="str">
+        <v>linda.johnson@company.com</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-04-09</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Thomas Rodriguez</v>
+      </c>
+      <c r="B13" t="str">
+        <v>thomas.rodriguez@company.com</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-08-02</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Robert Smith</v>
+      </c>
+      <c r="B14" t="str">
+        <v>robert.smith@company.com</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-03-19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Karen Martinez</v>
+      </c>
+      <c r="B15" t="str">
+        <v>karen.martinez@company.com</v>
+      </c>
+      <c r="C15" t="str">
         <v>Marketing</v>
       </c>
-      <c r="G3" t="str">
-        <v>Happy Work Anniversary Sang! Thank you for your dedication!</v>
+      <c r="D15" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-09-07</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Joseph Davis</v>
+      </c>
+      <c r="B16" t="str">
+        <v>joseph.davis@company.com</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-10-18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Robert Williams</v>
+      </c>
+      <c r="B17" t="str">
+        <v>robert.williams@company.com</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2026-05-17</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Elizabeth Davis</v>
+      </c>
+      <c r="B18" t="str">
+        <v>elizabeth.davis@company.com</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2026-03-20</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Barbara Moore</v>
+      </c>
+      <c r="B19" t="str">
+        <v>barbara.moore@company.com</v>
+      </c>
+      <c r="C19" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-05-27</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>James Rodriguez</v>
+      </c>
+      <c r="B20" t="str">
+        <v>james.rodriguez@company.com</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-12-15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Richard Taylor</v>
+      </c>
+      <c r="B21" t="str">
+        <v>richard.taylor@company.com</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-03-12</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Linda Smith</v>
+      </c>
+      <c r="B22" t="str">
+        <v>linda.smith@company.com</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2026-03-19</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>John Lopez</v>
+      </c>
+      <c r="B23" t="str">
+        <v>john.lopez@company.com</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2026-07-19</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Barbara Martin</v>
+      </c>
+      <c r="B24" t="str">
+        <v>barbara.martin@company.com</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2026-02-26</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Michael Lopez</v>
+      </c>
+      <c r="B25" t="str">
+        <v>michael.lopez@company.com</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2026-11-04</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Robert Johnson</v>
+      </c>
+      <c r="B26" t="str">
+        <v>robert.johnson@company.com</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2026-10-29</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Richard Martinez</v>
+      </c>
+      <c r="B27" t="str">
+        <v>richard.martinez@company.com</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2026-09-27</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>John Miller</v>
+      </c>
+      <c r="B28" t="str">
+        <v>john.miller@company.com</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2026-04-08</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Mary Gonzalez</v>
+      </c>
+      <c r="B29" t="str">
+        <v>mary.gonzalez@company.com</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2026-03-21</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>William Williams</v>
+      </c>
+      <c r="B30" t="str">
+        <v>william.williams@company.com</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2026-03-22</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Sarah Thomas</v>
+      </c>
+      <c r="B31" t="str">
+        <v>sarah.thomas@company.com</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2026-04-05</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Barbara Williams</v>
+      </c>
+      <c r="B32" t="str">
+        <v>barbara.williams@company.com</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2026-03-12</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Richard Davis</v>
+      </c>
+      <c r="B33" t="str">
+        <v>richard.davis@company.com</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2026-05-04</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Jennifer Wilson</v>
+      </c>
+      <c r="B34" t="str">
+        <v>jennifer.wilson@company.com</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2026-08-27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>John Thomas</v>
+      </c>
+      <c r="B35" t="str">
+        <v>john.thomas@company.com</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2026-04-05</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Michael Brown</v>
+      </c>
+      <c r="B36" t="str">
+        <v>michael.brown@company.com</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2026-10-08</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Thomas Hernandez</v>
+      </c>
+      <c r="B37" t="str">
+        <v>thomas.hernandez@company.com</v>
+      </c>
+      <c r="C37" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2026-11-10</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Karen Lopez</v>
+      </c>
+      <c r="B38" t="str">
+        <v>karen.lopez@company.com</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2026-11-05</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Susan Miller</v>
+      </c>
+      <c r="B39" t="str">
+        <v>susan.miller@company.com</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2026-05-22</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Linda Miller</v>
+      </c>
+      <c r="B40" t="str">
+        <v>linda.miller@company.com</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2026-01-10</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Linda Williams</v>
+      </c>
+      <c r="B41" t="str">
+        <v>linda.williams@company.com</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E41" t="str">
+        <v>2026-03-23</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>James Johnson</v>
+      </c>
+      <c r="B42" t="str">
+        <v>james.johnson@company.com</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E42" t="str">
+        <v>2026-09-16</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Jennifer Rodriguez</v>
+      </c>
+      <c r="B43" t="str">
+        <v>jennifer.rodriguez@company.com</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E43" t="str">
+        <v>2026-03-20</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Jennifer Garcia</v>
+      </c>
+      <c r="B44" t="str">
+        <v>jennifer.garcia@company.com</v>
+      </c>
+      <c r="C44" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2026-07-28</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>James Martinez</v>
+      </c>
+      <c r="B45" t="str">
+        <v>james.martinez@company.com</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E45" t="str">
+        <v>2026-10-14</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Linda Smith</v>
+      </c>
+      <c r="B46" t="str">
+        <v>linda.smith@company.com</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Sales</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2026-03-20</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Charles Gonzalez</v>
+      </c>
+      <c r="B47" t="str">
+        <v>charles.gonzalez@company.com</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2026-07-29</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Patricia Garcia</v>
+      </c>
+      <c r="B48" t="str">
+        <v>patricia.garcia@company.com</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Product</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2026-07-08</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Thomas Davis</v>
+      </c>
+      <c r="B49" t="str">
+        <v>thomas.davis@company.com</v>
+      </c>
+      <c r="C49" t="str">
+        <v>HR</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2026-03-30</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Robert Taylor</v>
+      </c>
+      <c r="B50" t="str">
+        <v>robert.taylor@company.com</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Design</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Work Anniversary</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2026-02-19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Jessica Davis</v>
+      </c>
+      <c r="B51" t="str">
+        <v>jessica.davis@company.com</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Engineering</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Birthday</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2026-10-17</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>